<commit_message>
Post Update 1: Added Redis Distributed Cache
</commit_message>
<xml_diff>
--- a/PMS/tests/test-assets/project-list/no_existing.xlsx
+++ b/PMS/tests/test-assets/project-list/no_existing.xlsx
@@ -34,22 +34,22 @@
     <t xml:space="preserve">Supervisor Email</t>
   </si>
   <si>
-    <t xml:space="preserve">ingest-project-1</t>
+    <t xml:space="preserve">E-Voting Blockchain System</t>
   </si>
   <si>
     <t xml:space="preserve">This is a ingested project</t>
   </si>
   <si>
-    <t xml:space="preserve">userB_student1@uni.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">userB_supervisor1@uni.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ingest-project-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">userB_student2@uni.com</t>
+    <t xml:space="preserve">student@uni.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supervisor@uni.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Management System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">student2@uni.com</t>
   </si>
 </sst>
 </file>
@@ -274,7 +274,7 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="27.26"/>
@@ -324,9 +324,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="userB_student1@uni.com"/>
-    <hyperlink ref="D2" r:id="rId2" display="userB_supervisor1@uni.com"/>
-    <hyperlink ref="D3" r:id="rId3" display="userB_supervisor1@uni.com"/>
+    <hyperlink ref="C2" r:id="rId1" display="student@uni.com"/>
+    <hyperlink ref="D2" r:id="rId2" display="supervisor@uni.com"/>
+    <hyperlink ref="C3" r:id="rId3" display="student2@uni.com"/>
+    <hyperlink ref="D3" r:id="rId4" display="supervisor@uni.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>